<commit_message>
Refactor Docker Compose files to rename upload_tasks volume to specific service volumes (wtchk_upload_tasks, wtcmy_upload_tasks, wtctw_upload_tasks) and enhance store data retrieval in the backend by returning structured StoreResponse objects with additional fields. Update background task processing to include cls_score and improve error handling for AI analysis tasks.
</commit_message>
<xml_diff>
--- a/backend/upload_tasks/example.xlsx
+++ b/backend/upload_tasks/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fktse\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmytse/Documents/CLSense-Backend/backend/upload_tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F655DD10-85AC-484F-BD68-F0C1C711D69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9095FA58-338C-7C4B-9D96-13B687C4ACAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7410" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{16151918-4ABF-4074-9B3A-A30577719F62}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="34200" windowHeight="19800" xr2:uid="{16151918-4ABF-4074-9B3A-A30577719F62}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>store_id</t>
   </si>
@@ -49,6 +49,9 @@
   <si>
     <t>店員態度很友善</t>
   </si>
+  <si>
+    <t>cls_score</t>
+  </si>
 </sst>
 </file>
 
@@ -58,14 +61,14 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
@@ -102,7 +105,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -118,7 +121,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -434,13 +437,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0844A3E6-8244-46CA-AA59-601935D4D1F8}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -450,8 +454,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>3202</v>
       </c>
@@ -461,6 +468,9 @@
       <c r="C2" s="1">
         <v>45872.014421296299</v>
       </c>
+      <c r="D2">
+        <v>1.2</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -469,12 +479,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7fd18732-2772-474e-a6da-6ca98635c5de" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -666,17 +675,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7fd18732-2772-474e-a6da-6ca98635c5de" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CB984FD-5B24-4BD3-99A7-A0216847885C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3A82D52-65E5-4554-9C2E-A982B2B10B26}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7fd18732-2772-474e-a6da-6ca98635c5de"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -700,17 +718,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3A82D52-65E5-4554-9C2E-A982B2B10B26}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CB984FD-5B24-4BD3-99A7-A0216847885C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7fd18732-2772-474e-a6da-6ca98635c5de"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>